<commit_message>
fix: consolidacao por SKU no top produtos
</commit_message>
<xml_diff>
--- a/data_external/vendas-tiktok.xlsx
+++ b/data_external/vendas-tiktok.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31834943-ECDF-41C7-98F4-D661A0542B78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DD3C208-737F-4569-A5C0-8BCDC1602E65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35640" yWindow="1860" windowWidth="22890" windowHeight="12615" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32205" yWindow="0" windowWidth="28155" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="OrderSKUList" sheetId="2" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3893" uniqueCount="1685">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3321" uniqueCount="1462">
   <si>
     <t>Order ID</t>
   </si>
@@ -4594,730 +4594,6 @@
 (+55)129******24
 ******************** ** **************** ********************
 Caraguatatuba, SP
-********
-Brasil</t>
-  </si>
-  <si>
-    <t>583719900735964534</t>
-  </si>
-  <si>
-    <t>1194272689855694198</t>
-  </si>
-  <si>
-    <t>1735194654563141106</t>
-  </si>
-  <si>
-    <t>DPX4901922276</t>
-  </si>
-  <si>
-    <t>Kit 2 Air Gun - 6 Dardo E 1 Alvo Brinquedo Presente</t>
-  </si>
-  <si>
-    <t>Detonadores e armas de brinquedo</t>
-  </si>
-  <si>
-    <t>BRL 45,15</t>
-  </si>
-  <si>
-    <t>BRL 45,95</t>
-  </si>
-  <si>
-    <t>04/27/2026 2:49:17 AM</t>
-  </si>
-  <si>
-    <t>04/27/2026 2:51:46 AM</t>
-  </si>
-  <si>
-    <t>04/27/2026 12:50:43 PM</t>
-  </si>
-  <si>
-    <t>3320086385424</t>
-  </si>
-  <si>
-    <t>henrique.nunes73</t>
-  </si>
-  <si>
-    <t>11716083737</t>
-  </si>
-  <si>
-    <t>FERNANDO HENRIQUE MACARIO</t>
-  </si>
-  <si>
-    <t>Henrique Nunes</t>
-  </si>
-  <si>
-    <t>(+55)249******34</t>
-  </si>
-  <si>
-    <t>rua alameda das revuadas</t>
-  </si>
-  <si>
-    <t>213</t>
-  </si>
-  <si>
-    <t>Bela vista</t>
-  </si>
-  <si>
-    <t>Paraíba do Sul</t>
-  </si>
-  <si>
-    <t>25850000</t>
-  </si>
-  <si>
-    <t>Henrique Nunes
-(+55)249******34
-rua alameda das revuadas 213 Bela vista casa
-Paraíba do Sul, RJ
-25850000
-Brasil</t>
-  </si>
-  <si>
-    <t>583716824348592069</t>
-  </si>
-  <si>
-    <t>1194245028078716869</t>
-  </si>
-  <si>
-    <t>04/26/2026 11:12:25 PM</t>
-  </si>
-  <si>
-    <t>04/26/2026 11:12:48 PM</t>
-  </si>
-  <si>
-    <t>04/27/2026 11:50:51 AM</t>
-  </si>
-  <si>
-    <t>3320080384875</t>
-  </si>
-  <si>
-    <t>_alexandersabino</t>
-  </si>
-  <si>
-    <t>18805790737</t>
-  </si>
-  <si>
-    <t>ALEXANDER SABINO INOCENTE</t>
-  </si>
-  <si>
-    <t>Alexander Sabino inocente</t>
-  </si>
-  <si>
-    <t>(+55)289******65</t>
-  </si>
-  <si>
-    <t>Rua Fernando Umlauf</t>
-  </si>
-  <si>
-    <t>192</t>
-  </si>
-  <si>
-    <t>Avaí</t>
-  </si>
-  <si>
-    <t>Guaramirim</t>
-  </si>
-  <si>
-    <t>89272014</t>
-  </si>
-  <si>
-    <t>Alexander Sabino inocente
-(+55)289******65
-Rua Fernando Umlauf 192 Avaí Casa
-Guaramirim, SC
-89272014
-Brasil</t>
-  </si>
-  <si>
-    <t>583713979232454417</t>
-  </si>
-  <si>
-    <t>1194215017126987537</t>
-  </si>
-  <si>
-    <t>04/26/2026 3:30:04 PM</t>
-  </si>
-  <si>
-    <t>04/26/2026 3:32:05 PM</t>
-  </si>
-  <si>
-    <t>04/27/2026 11:49:26 AM</t>
-  </si>
-  <si>
-    <t>3320084387116</t>
-  </si>
-  <si>
-    <t>sol.costaaa</t>
-  </si>
-  <si>
-    <t>18213942833</t>
-  </si>
-  <si>
-    <t>SOLANGE DA COSTA DE GOIS</t>
-  </si>
-  <si>
-    <t>(+55)199******60</t>
-  </si>
-  <si>
-    <t>Rua Doutor Alberto Ferraz Abreu</t>
-  </si>
-  <si>
-    <t>88</t>
-  </si>
-  <si>
-    <t>Jardim Nossa Senhora Auxiliadora</t>
-  </si>
-  <si>
-    <t>ap 102</t>
-  </si>
-  <si>
-    <t>Campinas</t>
-  </si>
-  <si>
-    <t>13075340</t>
-  </si>
-  <si>
-    <t>sol.costaaa
-(+55)199******60
-Rua Doutor Alberto Ferraz Abreu 88 Jardim Nossa Senhora Auxiliadora ap 102
-Campinas, SP
-13075340
-Brasil</t>
-  </si>
-  <si>
-    <t>583713928085669440</t>
-  </si>
-  <si>
-    <t>1194214766565033536</t>
-  </si>
-  <si>
-    <t>BRL 0,15</t>
-  </si>
-  <si>
-    <t>BRL 45,00</t>
-  </si>
-  <si>
-    <t>04/26/2026 3:19:00 PM</t>
-  </si>
-  <si>
-    <t>04/26/2026 3:21:59 PM</t>
-  </si>
-  <si>
-    <t>04/27/2026 11:46:55 AM</t>
-  </si>
-  <si>
-    <t>3320080383811</t>
-  </si>
-  <si>
-    <t>jonh_bala_2.0</t>
-  </si>
-  <si>
-    <t>53694090134</t>
-  </si>
-  <si>
-    <t>ALEXANDRE ALBERTO RODRIGUES DE FREITAS</t>
-  </si>
-  <si>
-    <t>alexandre alberto</t>
-  </si>
-  <si>
-    <t>(+55)619******28</t>
-  </si>
-  <si>
-    <t>Quadra CSB 4</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>Taguatinga Sul</t>
-  </si>
-  <si>
-    <t>102</t>
-  </si>
-  <si>
-    <t>72015545</t>
-  </si>
-  <si>
-    <t>alexandre alberto
-(+55)619******28
-Quadra CSB 4 4 Taguatinga Sul 102
-Brasília, DF
-72015545
-Brasil</t>
-  </si>
-  <si>
-    <t>583700151427434087</t>
-  </si>
-  <si>
-    <t>BRL 47,15</t>
-  </si>
-  <si>
-    <t>04/25/2026 9:09:54 PM</t>
-  </si>
-  <si>
-    <t>04/25/2026 9:11:31 PM</t>
-  </si>
-  <si>
-    <t>delson.rodrigues50</t>
-  </si>
-  <si>
-    <t>01098049616</t>
-  </si>
-  <si>
-    <t>MARIA CONCEICAO DOS REIS</t>
-  </si>
-  <si>
-    <t>D***** R******** d* M***</t>
-  </si>
-  <si>
-    <t>(+55)359******71</t>
-  </si>
-  <si>
-    <t>Alfenas</t>
-  </si>
-  <si>
-    <t>D***** R******** d* M***
-(+55)359******71
-************ *** ******************* ****
-Alfenas, MG
-********
-Brasil</t>
-  </si>
-  <si>
-    <t>583700129123698279</t>
-  </si>
-  <si>
-    <t>04/25/2026 9:09:02 PM</t>
-  </si>
-  <si>
-    <t>04/25/2026 9:09:36 PM</t>
-  </si>
-  <si>
-    <t>583686411103274533</t>
-  </si>
-  <si>
-    <t>1194041094445434405</t>
-  </si>
-  <si>
-    <t>1735164039157614066</t>
-  </si>
-  <si>
-    <t>DPX6895184061</t>
-  </si>
-  <si>
-    <t>Bengala Retrátil Dobrável Ajustável Idosos Deficiente Tip -</t>
-  </si>
-  <si>
-    <t>Equipamento de ginástica aquática</t>
-  </si>
-  <si>
-    <t>BRL 118,09</t>
-  </si>
-  <si>
-    <t>BRL 4,95</t>
-  </si>
-  <si>
-    <t>BRL 108,14</t>
-  </si>
-  <si>
-    <t>04/24/2026 11:40:09 PM</t>
-  </si>
-  <si>
-    <t>04/24/2026 11:41:49 PM</t>
-  </si>
-  <si>
-    <t>04/27/2026 11:51:49 AM</t>
-  </si>
-  <si>
-    <t>3320085380170</t>
-  </si>
-  <si>
-    <t>lurdes.cabrera5</t>
-  </si>
-  <si>
-    <t>00958224960</t>
-  </si>
-  <si>
-    <t>MARIA LOURDES CABRERA ARANDA</t>
-  </si>
-  <si>
-    <t>Lurdes Cabrera</t>
-  </si>
-  <si>
-    <t>(+55)459******33</t>
-  </si>
-  <si>
-    <t>avenida Florianópolis</t>
-  </si>
-  <si>
-    <t>427</t>
-  </si>
-  <si>
-    <t>klp</t>
-  </si>
-  <si>
-    <t>Foz do Iguaçu</t>
-  </si>
-  <si>
-    <t>85868090</t>
-  </si>
-  <si>
-    <t>Lurdes Cabrera
-(+55)459******33
-avenida Florianópolis 427 klp casa
-Foz do Iguaçu, PR
-85868090
-Brasil</t>
-  </si>
-  <si>
-    <t>583653579411130222</t>
-  </si>
-  <si>
-    <t>1193791632311355246</t>
-  </si>
-  <si>
-    <t>1735168384624133618</t>
-  </si>
-  <si>
-    <t>DPX5629937500</t>
-  </si>
-  <si>
-    <t>Suporte Capa Telefone Celular Chuveiro Banho A Prova -</t>
-  </si>
-  <si>
-    <t>Suportes para telefone</t>
-  </si>
-  <si>
-    <t>BRL 61,46</t>
-  </si>
-  <si>
-    <t>BRL 1,36</t>
-  </si>
-  <si>
-    <t>BRL 11,06</t>
-  </si>
-  <si>
-    <t>BRL 49,04</t>
-  </si>
-  <si>
-    <t>Apple Pay</t>
-  </si>
-  <si>
-    <t>04/22/2026 7:32:01 PM</t>
-  </si>
-  <si>
-    <t>04/22/2026 7:32:07 PM</t>
-  </si>
-  <si>
-    <t>04/24/2026 11:57:33 AM</t>
-  </si>
-  <si>
-    <t>3320017388034</t>
-  </si>
-  <si>
-    <t>carol_gco11</t>
-  </si>
-  <si>
-    <t>01560507659</t>
-  </si>
-  <si>
-    <t>CAROLINA GUIMARAES CAMPOS DE OLIVEIRA</t>
-  </si>
-  <si>
-    <t>Cristiana Guimarães</t>
-  </si>
-  <si>
-    <t>(+55)379******96</t>
-  </si>
-  <si>
-    <t>Rua Mares de Montanhas</t>
-  </si>
-  <si>
-    <t>1265</t>
-  </si>
-  <si>
-    <t>Vale dos Cristais</t>
-  </si>
-  <si>
-    <t>Nova Lima</t>
-  </si>
-  <si>
-    <t>34008056</t>
-  </si>
-  <si>
-    <t>Cristiana Guimarães
-(+55)379******96
-Rua Mares de Montanhas 1265 Vale dos Cristais Rua Mares de Montanhas
-Nova Lima, MG
-34008056
-Brasil</t>
-  </si>
-  <si>
-    <t>NF-e error</t>
-  </si>
-  <si>
-    <t>583623577445303727</t>
-  </si>
-  <si>
-    <t>1193566513186899375</t>
-  </si>
-  <si>
-    <t>1735185763935094258</t>
-  </si>
-  <si>
-    <t>DPX7356783327</t>
-  </si>
-  <si>
-    <t>Espada Luminosa Grande Samurai -</t>
-  </si>
-  <si>
-    <t>Modelos e veículos de brinquedo</t>
-  </si>
-  <si>
-    <t>BRL 60,88</t>
-  </si>
-  <si>
-    <t>BRL 9,89</t>
-  </si>
-  <si>
-    <t>BRL 14,13</t>
-  </si>
-  <si>
-    <t>BRL 36,86</t>
-  </si>
-  <si>
-    <t>BRL 7,50</t>
-  </si>
-  <si>
-    <t>BRL 27,50</t>
-  </si>
-  <si>
-    <t>BRL 20,00</t>
-  </si>
-  <si>
-    <t>BRL 44,36</t>
-  </si>
-  <si>
-    <t>04/20/2026 7:32:17 PM</t>
-  </si>
-  <si>
-    <t>04/23/2026 12:34:25 PM</t>
-  </si>
-  <si>
-    <t>3320084375097</t>
-  </si>
-  <si>
-    <t>0.4</t>
-  </si>
-  <si>
-    <t>tiagoaugusto1357911</t>
-  </si>
-  <si>
-    <t>00863924336</t>
-  </si>
-  <si>
-    <t>MARTA CIBELLI BORGES PEREIRA</t>
-  </si>
-  <si>
-    <t>Marta</t>
-  </si>
-  <si>
-    <t>(+55)999******56</t>
-  </si>
-  <si>
-    <t>travessa Siqueira Campos</t>
-  </si>
-  <si>
-    <t>112</t>
-  </si>
-  <si>
-    <t>Passagem Franca</t>
-  </si>
-  <si>
-    <t>65680000</t>
-  </si>
-  <si>
-    <t>Marta
-(+55)999******56
-travessa Siqueira Campos 112 centro travessa Siqueira Campos
-Passagem Franca, MA
-65680000
-Brasil</t>
-  </si>
-  <si>
-    <t>583579397031888154</t>
-  </si>
-  <si>
-    <t>1193244865603339546</t>
-  </si>
-  <si>
-    <t>1735138280380663282</t>
-  </si>
-  <si>
-    <t>DPX4131268835</t>
-  </si>
-  <si>
-    <t>Corda De Pular Crossfit Speed Rope Rolamento 3M Cabo De Aço</t>
-  </si>
-  <si>
-    <t>Cordas de pular</t>
-  </si>
-  <si>
-    <t>BRL 59,45</t>
-  </si>
-  <si>
-    <t>BRL 1,52</t>
-  </si>
-  <si>
-    <t>BRL 8,91</t>
-  </si>
-  <si>
-    <t>BRL 49,02</t>
-  </si>
-  <si>
-    <t>BRL 16,30</t>
-  </si>
-  <si>
-    <t>BRL 65,32</t>
-  </si>
-  <si>
-    <t>04/17/2026 8:24:13 PM</t>
-  </si>
-  <si>
-    <t>04/17/2026 8:24:57 PM</t>
-  </si>
-  <si>
-    <t>04/23/2026 12:24:30 PM</t>
-  </si>
-  <si>
-    <t>3320093371832</t>
-  </si>
-  <si>
-    <t>0.7</t>
-  </si>
-  <si>
-    <t>scovslovs</t>
-  </si>
-  <si>
-    <t>78854237191</t>
-  </si>
-  <si>
-    <t>RENATO ARANTES DE ARAUJO</t>
-  </si>
-  <si>
-    <t>Renato Arantes de Araújo</t>
-  </si>
-  <si>
-    <t>(+55)629******15</t>
-  </si>
-  <si>
-    <t>Av Sebastião Fleury Curado</t>
-  </si>
-  <si>
-    <t>250</t>
-  </si>
-  <si>
-    <t>Banco do Brasil</t>
-  </si>
-  <si>
-    <t>Goiás</t>
-  </si>
-  <si>
-    <t>76600000</t>
-  </si>
-  <si>
-    <t>Renato Arantes de Araújo
-(+55)629******15
-Av Sebastião Fleury Curado 250 Centro Banco do Brasil
-Goiás, GO
-76600000
-Brasil</t>
-  </si>
-  <si>
-    <t>583564264957445402</t>
-  </si>
-  <si>
-    <t>BRL 50,54</t>
-  </si>
-  <si>
-    <t>BRL 66,84</t>
-  </si>
-  <si>
-    <t>04/16/2026 6:54:55 PM</t>
-  </si>
-  <si>
-    <t>04/17/2026 6:54:58 PM</t>
-  </si>
-  <si>
-    <t>R***** A****** d* A*****</t>
-  </si>
-  <si>
-    <t>R***** A****** d* A*****
-(+55)629******15
-************************** *** ****** ***************
-Goiás, GO
-********
-Brasil</t>
-  </si>
-  <si>
-    <t>583559683789718880</t>
-  </si>
-  <si>
-    <t>1735138550063924722</t>
-  </si>
-  <si>
-    <t>DPX9722332548</t>
-  </si>
-  <si>
-    <t>Jogo De Cartas Uno No Mercy Bordô Inglês, Portugês, Espan -</t>
-  </si>
-  <si>
-    <t>Jogos de cartas</t>
-  </si>
-  <si>
-    <t>BRL 51,44</t>
-  </si>
-  <si>
-    <t>BRL 7,71</t>
-  </si>
-  <si>
-    <t>BRL 43,73</t>
-  </si>
-  <si>
-    <t>BRL 48,23</t>
-  </si>
-  <si>
-    <t>04/16/2026 9:38:20 AM</t>
-  </si>
-  <si>
-    <t>04/16/2026 9:50:12 AM</t>
-  </si>
-  <si>
-    <t>my_name_is_brun0</t>
-  </si>
-  <si>
-    <t>61941826369</t>
-  </si>
-  <si>
-    <t>IVANBRUNO BARROS PIRES</t>
-  </si>
-  <si>
-    <t>I******** B***** P****</t>
-  </si>
-  <si>
-    <t>(+55)858*****30</t>
-  </si>
-  <si>
-    <t>******************************</t>
-  </si>
-  <si>
-    <t>Fortaleza</t>
-  </si>
-  <si>
-    <t>I******** B***** P****
-(+55)858*****30
-********************** **** ****************** ******************************
-Fortaleza, CE
 ********
 Brasil</t>
   </si>
@@ -5736,7 +5012,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BF80"/>
+  <dimension ref="A1:BF68"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -5923,109 +5199,109 @@
     </row>
     <row r="2" spans="1:58" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>1650</v>
+        <v>1427</v>
       </c>
       <c r="B2" t="s">
-        <v>1651</v>
+        <v>1428</v>
       </c>
       <c r="C2" t="s">
-        <v>1652</v>
+        <v>1429</v>
       </c>
       <c r="E2" t="s">
-        <v>1653</v>
+        <v>1430</v>
       </c>
       <c r="G2" t="s">
-        <v>1654</v>
+        <v>1431</v>
       </c>
       <c r="H2" t="s">
-        <v>1655</v>
+        <v>1432</v>
       </c>
       <c r="I2" t="s">
-        <v>1656</v>
+        <v>1433</v>
       </c>
       <c r="J2" t="s">
-        <v>1657</v>
+        <v>1434</v>
       </c>
       <c r="K2" t="s">
-        <v>1658</v>
+        <v>1435</v>
       </c>
       <c r="L2" t="s">
-        <v>1659</v>
+        <v>1436</v>
       </c>
       <c r="M2" t="s">
-        <v>1660</v>
+        <v>1437</v>
       </c>
       <c r="N2" t="s">
-        <v>1661</v>
+        <v>1438</v>
       </c>
       <c r="O2" t="s">
-        <v>1662</v>
+        <v>1439</v>
       </c>
       <c r="P2" t="s">
-        <v>1663</v>
+        <v>1440</v>
       </c>
       <c r="Q2" t="s">
-        <v>1664</v>
+        <v>1441</v>
       </c>
       <c r="R2" t="s">
-        <v>1665</v>
+        <v>1442</v>
       </c>
       <c r="S2" t="s">
-        <v>1666</v>
+        <v>1443</v>
       </c>
       <c r="T2" t="s">
-        <v>1667</v>
+        <v>1444</v>
       </c>
       <c r="U2" t="s">
-        <v>1668</v>
+        <v>1445</v>
       </c>
       <c r="V2" t="s">
-        <v>1669</v>
+        <v>1446</v>
       </c>
       <c r="W2" t="s">
-        <v>1670</v>
+        <v>1447</v>
       </c>
       <c r="X2" t="s">
-        <v>1671</v>
+        <v>1448</v>
       </c>
       <c r="Y2" t="s">
-        <v>1672</v>
+        <v>1449</v>
       </c>
       <c r="Z2" t="s">
-        <v>1673</v>
+        <v>1450</v>
       </c>
       <c r="AA2" t="s">
-        <v>1674</v>
+        <v>1451</v>
       </c>
       <c r="AB2" t="s">
-        <v>1675</v>
+        <v>1452</v>
       </c>
       <c r="AC2" t="s">
-        <v>1676</v>
+        <v>1453</v>
       </c>
       <c r="AD2" t="s">
-        <v>1677</v>
+        <v>1454</v>
       </c>
       <c r="AE2" t="s">
-        <v>1678</v>
+        <v>1455</v>
       </c>
       <c r="AF2" t="s">
-        <v>1679</v>
+        <v>1456</v>
       </c>
       <c r="AG2" t="s">
-        <v>1680</v>
+        <v>1457</v>
       </c>
       <c r="AH2" t="s">
-        <v>1681</v>
+        <v>1458</v>
       </c>
       <c r="AK2" t="s">
-        <v>1682</v>
+        <v>1459</v>
       </c>
       <c r="AM2" t="s">
-        <v>1683</v>
+        <v>1460</v>
       </c>
       <c r="AO2" t="s">
-        <v>1684</v>
+        <v>1461</v>
       </c>
     </row>
     <row r="3" spans="1:58" x14ac:dyDescent="0.35">
@@ -15842,1746 +15118,6 @@
       </c>
       <c r="BC68" t="s">
         <v>1426</v>
-      </c>
-    </row>
-    <row r="69" spans="1:58" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
-        <v>1427</v>
-      </c>
-      <c r="B69" t="s">
-        <v>1428</v>
-      </c>
-      <c r="C69" t="s">
-        <v>60</v>
-      </c>
-      <c r="D69" t="s">
-        <v>61</v>
-      </c>
-      <c r="F69" t="s">
-        <v>62</v>
-      </c>
-      <c r="G69" t="s">
-        <v>1429</v>
-      </c>
-      <c r="H69" t="s">
-        <v>1430</v>
-      </c>
-      <c r="I69" t="s">
-        <v>1431</v>
-      </c>
-      <c r="J69" t="s">
-        <v>176</v>
-      </c>
-      <c r="K69" t="s">
-        <v>1432</v>
-      </c>
-      <c r="L69" t="s">
-        <v>68</v>
-      </c>
-      <c r="M69" t="s">
-        <v>69</v>
-      </c>
-      <c r="N69" t="s">
-        <v>1433</v>
-      </c>
-      <c r="O69" t="s">
-        <v>1433</v>
-      </c>
-      <c r="P69" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q69" t="s">
-        <v>71</v>
-      </c>
-      <c r="R69" t="s">
-        <v>1433</v>
-      </c>
-      <c r="S69" t="s">
-        <v>74</v>
-      </c>
-      <c r="T69" t="s">
-        <v>75</v>
-      </c>
-      <c r="U69" t="s">
-        <v>71</v>
-      </c>
-      <c r="V69" t="s">
-        <v>76</v>
-      </c>
-      <c r="X69" t="s">
-        <v>1434</v>
-      </c>
-      <c r="Y69" t="s">
-        <v>129</v>
-      </c>
-      <c r="AC69" t="s">
-        <v>1435</v>
-      </c>
-      <c r="AD69" t="s">
-        <v>1436</v>
-      </c>
-      <c r="AE69" t="s">
-        <v>1437</v>
-      </c>
-      <c r="AI69" t="s">
-        <v>82</v>
-      </c>
-      <c r="AJ69" t="s">
-        <v>97</v>
-      </c>
-      <c r="AK69" t="s">
-        <v>1438</v>
-      </c>
-      <c r="AL69" t="s">
-        <v>85</v>
-      </c>
-      <c r="AM69" t="s">
-        <v>86</v>
-      </c>
-      <c r="AN69" t="s">
-        <v>134</v>
-      </c>
-      <c r="AO69" t="s">
-        <v>88</v>
-      </c>
-      <c r="AP69" t="s">
-        <v>1439</v>
-      </c>
-      <c r="AQ69" t="s">
-        <v>1440</v>
-      </c>
-      <c r="AR69" t="s">
-        <v>1441</v>
-      </c>
-      <c r="AS69" t="s">
-        <v>1442</v>
-      </c>
-      <c r="AT69" t="s">
-        <v>1443</v>
-      </c>
-      <c r="AU69" t="s">
-        <v>1444</v>
-      </c>
-      <c r="AV69" t="s">
-        <v>1445</v>
-      </c>
-      <c r="AW69" t="s">
-        <v>1446</v>
-      </c>
-      <c r="AX69" t="s">
-        <v>582</v>
-      </c>
-      <c r="AY69" t="s">
-        <v>1447</v>
-      </c>
-      <c r="AZ69" t="s">
-        <v>97</v>
-      </c>
-      <c r="BA69" t="s">
-        <v>98</v>
-      </c>
-      <c r="BB69" t="s">
-        <v>1448</v>
-      </c>
-      <c r="BC69" t="s">
-        <v>1449</v>
-      </c>
-      <c r="BD69" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="70" spans="1:58" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
-        <v>1450</v>
-      </c>
-      <c r="B70" t="s">
-        <v>1451</v>
-      </c>
-      <c r="C70" t="s">
-        <v>60</v>
-      </c>
-      <c r="D70" t="s">
-        <v>61</v>
-      </c>
-      <c r="F70" t="s">
-        <v>62</v>
-      </c>
-      <c r="G70" t="s">
-        <v>1429</v>
-      </c>
-      <c r="H70" t="s">
-        <v>1430</v>
-      </c>
-      <c r="I70" t="s">
-        <v>1431</v>
-      </c>
-      <c r="J70" t="s">
-        <v>176</v>
-      </c>
-      <c r="K70" t="s">
-        <v>1432</v>
-      </c>
-      <c r="L70" t="s">
-        <v>68</v>
-      </c>
-      <c r="M70" t="s">
-        <v>69</v>
-      </c>
-      <c r="N70" t="s">
-        <v>1433</v>
-      </c>
-      <c r="O70" t="s">
-        <v>1433</v>
-      </c>
-      <c r="P70" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q70" t="s">
-        <v>71</v>
-      </c>
-      <c r="R70" t="s">
-        <v>1433</v>
-      </c>
-      <c r="S70" t="s">
-        <v>74</v>
-      </c>
-      <c r="T70" t="s">
-        <v>75</v>
-      </c>
-      <c r="U70" t="s">
-        <v>71</v>
-      </c>
-      <c r="V70" t="s">
-        <v>76</v>
-      </c>
-      <c r="X70" t="s">
-        <v>1434</v>
-      </c>
-      <c r="Y70" t="s">
-        <v>129</v>
-      </c>
-      <c r="AC70" t="s">
-        <v>1452</v>
-      </c>
-      <c r="AD70" t="s">
-        <v>1453</v>
-      </c>
-      <c r="AE70" t="s">
-        <v>1454</v>
-      </c>
-      <c r="AI70" t="s">
-        <v>82</v>
-      </c>
-      <c r="AJ70" t="s">
-        <v>97</v>
-      </c>
-      <c r="AK70" t="s">
-        <v>1455</v>
-      </c>
-      <c r="AL70" t="s">
-        <v>85</v>
-      </c>
-      <c r="AM70" t="s">
-        <v>86</v>
-      </c>
-      <c r="AN70" t="s">
-        <v>134</v>
-      </c>
-      <c r="AO70" t="s">
-        <v>88</v>
-      </c>
-      <c r="AP70" t="s">
-        <v>1456</v>
-      </c>
-      <c r="AQ70" t="s">
-        <v>1457</v>
-      </c>
-      <c r="AR70" t="s">
-        <v>1458</v>
-      </c>
-      <c r="AS70" t="s">
-        <v>1459</v>
-      </c>
-      <c r="AT70" t="s">
-        <v>1460</v>
-      </c>
-      <c r="AU70" t="s">
-        <v>1461</v>
-      </c>
-      <c r="AV70" t="s">
-        <v>1462</v>
-      </c>
-      <c r="AW70" t="s">
-        <v>1463</v>
-      </c>
-      <c r="AX70" t="s">
-        <v>115</v>
-      </c>
-      <c r="AY70" t="s">
-        <v>1464</v>
-      </c>
-      <c r="AZ70" t="s">
-        <v>489</v>
-      </c>
-      <c r="BA70" t="s">
-        <v>98</v>
-      </c>
-      <c r="BB70" t="s">
-        <v>1465</v>
-      </c>
-      <c r="BC70" t="s">
-        <v>1466</v>
-      </c>
-      <c r="BD70" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="71" spans="1:58" x14ac:dyDescent="0.35">
-      <c r="A71" t="s">
-        <v>1467</v>
-      </c>
-      <c r="B71" t="s">
-        <v>1468</v>
-      </c>
-      <c r="C71" t="s">
-        <v>60</v>
-      </c>
-      <c r="D71" t="s">
-        <v>61</v>
-      </c>
-      <c r="F71" t="s">
-        <v>62</v>
-      </c>
-      <c r="G71" t="s">
-        <v>1429</v>
-      </c>
-      <c r="H71" t="s">
-        <v>1430</v>
-      </c>
-      <c r="I71" t="s">
-        <v>1431</v>
-      </c>
-      <c r="J71" t="s">
-        <v>176</v>
-      </c>
-      <c r="K71" t="s">
-        <v>1432</v>
-      </c>
-      <c r="L71" t="s">
-        <v>68</v>
-      </c>
-      <c r="M71" t="s">
-        <v>69</v>
-      </c>
-      <c r="N71" t="s">
-        <v>1433</v>
-      </c>
-      <c r="O71" t="s">
-        <v>1433</v>
-      </c>
-      <c r="P71" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q71" t="s">
-        <v>71</v>
-      </c>
-      <c r="R71" t="s">
-        <v>1433</v>
-      </c>
-      <c r="S71" t="s">
-        <v>71</v>
-      </c>
-      <c r="T71" t="s">
-        <v>245</v>
-      </c>
-      <c r="U71" t="s">
-        <v>71</v>
-      </c>
-      <c r="V71" t="s">
-        <v>245</v>
-      </c>
-      <c r="X71" t="s">
-        <v>1433</v>
-      </c>
-      <c r="Y71" t="s">
-        <v>129</v>
-      </c>
-      <c r="AC71" t="s">
-        <v>1469</v>
-      </c>
-      <c r="AD71" t="s">
-        <v>1470</v>
-      </c>
-      <c r="AE71" t="s">
-        <v>1471</v>
-      </c>
-      <c r="AI71" t="s">
-        <v>82</v>
-      </c>
-      <c r="AJ71" t="s">
-        <v>97</v>
-      </c>
-      <c r="AK71" t="s">
-        <v>1472</v>
-      </c>
-      <c r="AL71" t="s">
-        <v>85</v>
-      </c>
-      <c r="AM71" t="s">
-        <v>86</v>
-      </c>
-      <c r="AN71" t="s">
-        <v>134</v>
-      </c>
-      <c r="AO71" t="s">
-        <v>88</v>
-      </c>
-      <c r="AP71" t="s">
-        <v>1473</v>
-      </c>
-      <c r="AQ71" t="s">
-        <v>1474</v>
-      </c>
-      <c r="AR71" t="s">
-        <v>1475</v>
-      </c>
-      <c r="AS71" t="s">
-        <v>1473</v>
-      </c>
-      <c r="AT71" t="s">
-        <v>1476</v>
-      </c>
-      <c r="AU71" t="s">
-        <v>1477</v>
-      </c>
-      <c r="AV71" t="s">
-        <v>1478</v>
-      </c>
-      <c r="AW71" t="s">
-        <v>1479</v>
-      </c>
-      <c r="AX71" t="s">
-        <v>1480</v>
-      </c>
-      <c r="AY71" t="s">
-        <v>1481</v>
-      </c>
-      <c r="AZ71" t="s">
-        <v>224</v>
-      </c>
-      <c r="BA71" t="s">
-        <v>98</v>
-      </c>
-      <c r="BB71" t="s">
-        <v>1482</v>
-      </c>
-      <c r="BC71" t="s">
-        <v>1483</v>
-      </c>
-      <c r="BD71" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="72" spans="1:58" x14ac:dyDescent="0.35">
-      <c r="A72" t="s">
-        <v>1484</v>
-      </c>
-      <c r="B72" t="s">
-        <v>1485</v>
-      </c>
-      <c r="C72" t="s">
-        <v>60</v>
-      </c>
-      <c r="D72" t="s">
-        <v>61</v>
-      </c>
-      <c r="F72" t="s">
-        <v>62</v>
-      </c>
-      <c r="G72" t="s">
-        <v>1429</v>
-      </c>
-      <c r="H72" t="s">
-        <v>1430</v>
-      </c>
-      <c r="I72" t="s">
-        <v>1431</v>
-      </c>
-      <c r="J72" t="s">
-        <v>176</v>
-      </c>
-      <c r="K72" t="s">
-        <v>1432</v>
-      </c>
-      <c r="L72" t="s">
-        <v>68</v>
-      </c>
-      <c r="M72" t="s">
-        <v>69</v>
-      </c>
-      <c r="N72" t="s">
-        <v>1433</v>
-      </c>
-      <c r="O72" t="s">
-        <v>1433</v>
-      </c>
-      <c r="P72" t="s">
-        <v>1486</v>
-      </c>
-      <c r="Q72" t="s">
-        <v>71</v>
-      </c>
-      <c r="R72" t="s">
-        <v>1487</v>
-      </c>
-      <c r="S72" t="s">
-        <v>71</v>
-      </c>
-      <c r="T72" t="s">
-        <v>245</v>
-      </c>
-      <c r="U72" t="s">
-        <v>71</v>
-      </c>
-      <c r="V72" t="s">
-        <v>245</v>
-      </c>
-      <c r="X72" t="s">
-        <v>1487</v>
-      </c>
-      <c r="Y72" t="s">
-        <v>129</v>
-      </c>
-      <c r="AC72" t="s">
-        <v>1488</v>
-      </c>
-      <c r="AD72" t="s">
-        <v>1489</v>
-      </c>
-      <c r="AE72" t="s">
-        <v>1490</v>
-      </c>
-      <c r="AI72" t="s">
-        <v>82</v>
-      </c>
-      <c r="AJ72" t="s">
-        <v>97</v>
-      </c>
-      <c r="AK72" t="s">
-        <v>1491</v>
-      </c>
-      <c r="AL72" t="s">
-        <v>85</v>
-      </c>
-      <c r="AM72" t="s">
-        <v>86</v>
-      </c>
-      <c r="AN72" t="s">
-        <v>134</v>
-      </c>
-      <c r="AO72" t="s">
-        <v>88</v>
-      </c>
-      <c r="AP72" t="s">
-        <v>1492</v>
-      </c>
-      <c r="AQ72" t="s">
-        <v>1493</v>
-      </c>
-      <c r="AR72" t="s">
-        <v>1494</v>
-      </c>
-      <c r="AS72" t="s">
-        <v>1495</v>
-      </c>
-      <c r="AT72" t="s">
-        <v>1496</v>
-      </c>
-      <c r="AU72" t="s">
-        <v>1497</v>
-      </c>
-      <c r="AV72" t="s">
-        <v>1498</v>
-      </c>
-      <c r="AW72" t="s">
-        <v>1499</v>
-      </c>
-      <c r="AX72" t="s">
-        <v>1500</v>
-      </c>
-      <c r="AY72" t="s">
-        <v>728</v>
-      </c>
-      <c r="AZ72" t="s">
-        <v>729</v>
-      </c>
-      <c r="BA72" t="s">
-        <v>98</v>
-      </c>
-      <c r="BB72" t="s">
-        <v>1501</v>
-      </c>
-      <c r="BC72" t="s">
-        <v>1502</v>
-      </c>
-      <c r="BD72" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="73" spans="1:58" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
-        <v>1503</v>
-      </c>
-      <c r="C73" t="s">
-        <v>350</v>
-      </c>
-      <c r="D73" t="s">
-        <v>350</v>
-      </c>
-      <c r="E73" t="s">
-        <v>351</v>
-      </c>
-      <c r="F73" t="s">
-        <v>62</v>
-      </c>
-      <c r="G73" t="s">
-        <v>1429</v>
-      </c>
-      <c r="H73" t="s">
-        <v>1430</v>
-      </c>
-      <c r="I73" t="s">
-        <v>1431</v>
-      </c>
-      <c r="J73" t="s">
-        <v>176</v>
-      </c>
-      <c r="K73" t="s">
-        <v>1432</v>
-      </c>
-      <c r="L73" t="s">
-        <v>68</v>
-      </c>
-      <c r="M73" t="s">
-        <v>68</v>
-      </c>
-      <c r="N73" t="s">
-        <v>1433</v>
-      </c>
-      <c r="O73" t="s">
-        <v>1433</v>
-      </c>
-      <c r="P73" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q73" t="s">
-        <v>71</v>
-      </c>
-      <c r="R73" t="s">
-        <v>1433</v>
-      </c>
-      <c r="S73" t="s">
-        <v>149</v>
-      </c>
-      <c r="T73" t="s">
-        <v>150</v>
-      </c>
-      <c r="U73" t="s">
-        <v>71</v>
-      </c>
-      <c r="V73" t="s">
-        <v>76</v>
-      </c>
-      <c r="X73" t="s">
-        <v>1504</v>
-      </c>
-      <c r="Y73" t="s">
-        <v>129</v>
-      </c>
-      <c r="Z73" t="s">
-        <v>1433</v>
-      </c>
-      <c r="AA73" t="s">
-        <v>360</v>
-      </c>
-      <c r="AB73" t="s">
-        <v>361</v>
-      </c>
-      <c r="AC73" t="s">
-        <v>1505</v>
-      </c>
-      <c r="AH73" t="s">
-        <v>1506</v>
-      </c>
-      <c r="AI73" t="s">
-        <v>82</v>
-      </c>
-      <c r="AJ73" t="s">
-        <v>97</v>
-      </c>
-      <c r="AL73" t="s">
-        <v>85</v>
-      </c>
-      <c r="AM73" t="s">
-        <v>86</v>
-      </c>
-      <c r="AN73" t="s">
-        <v>134</v>
-      </c>
-      <c r="AP73" t="s">
-        <v>1507</v>
-      </c>
-      <c r="AQ73" t="s">
-        <v>1508</v>
-      </c>
-      <c r="AR73" t="s">
-        <v>1509</v>
-      </c>
-      <c r="AS73" t="s">
-        <v>1510</v>
-      </c>
-      <c r="AT73" t="s">
-        <v>1511</v>
-      </c>
-      <c r="AU73" t="s">
-        <v>430</v>
-      </c>
-      <c r="AV73" t="s">
-        <v>370</v>
-      </c>
-      <c r="AW73" t="s">
-        <v>595</v>
-      </c>
-      <c r="AX73" t="s">
-        <v>487</v>
-      </c>
-      <c r="AY73" t="s">
-        <v>1512</v>
-      </c>
-      <c r="AZ73" t="s">
-        <v>166</v>
-      </c>
-      <c r="BA73" t="s">
-        <v>98</v>
-      </c>
-      <c r="BB73" t="s">
-        <v>373</v>
-      </c>
-      <c r="BC73" t="s">
-        <v>1513</v>
-      </c>
-    </row>
-    <row r="74" spans="1:58" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
-        <v>1514</v>
-      </c>
-      <c r="C74" t="s">
-        <v>350</v>
-      </c>
-      <c r="D74" t="s">
-        <v>350</v>
-      </c>
-      <c r="E74" t="s">
-        <v>351</v>
-      </c>
-      <c r="F74" t="s">
-        <v>62</v>
-      </c>
-      <c r="G74" t="s">
-        <v>1429</v>
-      </c>
-      <c r="H74" t="s">
-        <v>1430</v>
-      </c>
-      <c r="I74" t="s">
-        <v>1431</v>
-      </c>
-      <c r="J74" t="s">
-        <v>176</v>
-      </c>
-      <c r="K74" t="s">
-        <v>1432</v>
-      </c>
-      <c r="L74" t="s">
-        <v>68</v>
-      </c>
-      <c r="M74" t="s">
-        <v>68</v>
-      </c>
-      <c r="N74" t="s">
-        <v>1433</v>
-      </c>
-      <c r="O74" t="s">
-        <v>1433</v>
-      </c>
-      <c r="P74" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q74" t="s">
-        <v>71</v>
-      </c>
-      <c r="R74" t="s">
-        <v>1433</v>
-      </c>
-      <c r="S74" t="s">
-        <v>149</v>
-      </c>
-      <c r="T74" t="s">
-        <v>150</v>
-      </c>
-      <c r="U74" t="s">
-        <v>71</v>
-      </c>
-      <c r="V74" t="s">
-        <v>76</v>
-      </c>
-      <c r="X74" t="s">
-        <v>1504</v>
-      </c>
-      <c r="Y74" t="s">
-        <v>129</v>
-      </c>
-      <c r="Z74" t="s">
-        <v>1433</v>
-      </c>
-      <c r="AA74" t="s">
-        <v>360</v>
-      </c>
-      <c r="AB74" t="s">
-        <v>361</v>
-      </c>
-      <c r="AC74" t="s">
-        <v>1515</v>
-      </c>
-      <c r="AH74" t="s">
-        <v>1516</v>
-      </c>
-      <c r="AI74" t="s">
-        <v>82</v>
-      </c>
-      <c r="AJ74" t="s">
-        <v>97</v>
-      </c>
-      <c r="AL74" t="s">
-        <v>85</v>
-      </c>
-      <c r="AM74" t="s">
-        <v>86</v>
-      </c>
-      <c r="AN74" t="s">
-        <v>134</v>
-      </c>
-      <c r="AP74" t="s">
-        <v>1507</v>
-      </c>
-      <c r="AQ74" t="s">
-        <v>1508</v>
-      </c>
-      <c r="AR74" t="s">
-        <v>1509</v>
-      </c>
-      <c r="AS74" t="s">
-        <v>1510</v>
-      </c>
-      <c r="AT74" t="s">
-        <v>1511</v>
-      </c>
-      <c r="AU74" t="s">
-        <v>430</v>
-      </c>
-      <c r="AV74" t="s">
-        <v>370</v>
-      </c>
-      <c r="AW74" t="s">
-        <v>595</v>
-      </c>
-      <c r="AX74" t="s">
-        <v>487</v>
-      </c>
-      <c r="AY74" t="s">
-        <v>1512</v>
-      </c>
-      <c r="AZ74" t="s">
-        <v>166</v>
-      </c>
-      <c r="BA74" t="s">
-        <v>98</v>
-      </c>
-      <c r="BB74" t="s">
-        <v>373</v>
-      </c>
-      <c r="BC74" t="s">
-        <v>1513</v>
-      </c>
-    </row>
-    <row r="75" spans="1:58" x14ac:dyDescent="0.35">
-      <c r="A75" t="s">
-        <v>1517</v>
-      </c>
-      <c r="B75" t="s">
-        <v>1518</v>
-      </c>
-      <c r="C75" t="s">
-        <v>60</v>
-      </c>
-      <c r="D75" t="s">
-        <v>61</v>
-      </c>
-      <c r="F75" t="s">
-        <v>62</v>
-      </c>
-      <c r="G75" t="s">
-        <v>1519</v>
-      </c>
-      <c r="H75" t="s">
-        <v>1520</v>
-      </c>
-      <c r="I75" t="s">
-        <v>1521</v>
-      </c>
-      <c r="J75" t="s">
-        <v>176</v>
-      </c>
-      <c r="K75" t="s">
-        <v>1522</v>
-      </c>
-      <c r="L75" t="s">
-        <v>68</v>
-      </c>
-      <c r="M75" t="s">
-        <v>69</v>
-      </c>
-      <c r="N75" t="s">
-        <v>1523</v>
-      </c>
-      <c r="O75" t="s">
-        <v>1523</v>
-      </c>
-      <c r="P75" t="s">
-        <v>1524</v>
-      </c>
-      <c r="Q75" t="s">
-        <v>243</v>
-      </c>
-      <c r="R75" t="s">
-        <v>1525</v>
-      </c>
-      <c r="S75" t="s">
-        <v>71</v>
-      </c>
-      <c r="T75" t="s">
-        <v>75</v>
-      </c>
-      <c r="U75" t="s">
-        <v>71</v>
-      </c>
-      <c r="V75" t="s">
-        <v>75</v>
-      </c>
-      <c r="X75" t="s">
-        <v>1525</v>
-      </c>
-      <c r="Y75" t="s">
-        <v>129</v>
-      </c>
-      <c r="AC75" t="s">
-        <v>1526</v>
-      </c>
-      <c r="AD75" t="s">
-        <v>1527</v>
-      </c>
-      <c r="AE75" t="s">
-        <v>1528</v>
-      </c>
-      <c r="AI75" t="s">
-        <v>82</v>
-      </c>
-      <c r="AJ75" t="s">
-        <v>97</v>
-      </c>
-      <c r="AK75" t="s">
-        <v>1529</v>
-      </c>
-      <c r="AL75" t="s">
-        <v>85</v>
-      </c>
-      <c r="AM75" t="s">
-        <v>86</v>
-      </c>
-      <c r="AN75" t="s">
-        <v>87</v>
-      </c>
-      <c r="AO75" t="s">
-        <v>88</v>
-      </c>
-      <c r="AP75" t="s">
-        <v>1530</v>
-      </c>
-      <c r="AQ75" t="s">
-        <v>1531</v>
-      </c>
-      <c r="AR75" t="s">
-        <v>1532</v>
-      </c>
-      <c r="AS75" t="s">
-        <v>1533</v>
-      </c>
-      <c r="AT75" t="s">
-        <v>1534</v>
-      </c>
-      <c r="AU75" t="s">
-        <v>1535</v>
-      </c>
-      <c r="AV75" t="s">
-        <v>1536</v>
-      </c>
-      <c r="AW75" t="s">
-        <v>1537</v>
-      </c>
-      <c r="AX75" t="s">
-        <v>582</v>
-      </c>
-      <c r="AY75" t="s">
-        <v>1538</v>
-      </c>
-      <c r="AZ75" t="s">
-        <v>262</v>
-      </c>
-      <c r="BA75" t="s">
-        <v>98</v>
-      </c>
-      <c r="BB75" t="s">
-        <v>1539</v>
-      </c>
-      <c r="BC75" t="s">
-        <v>1540</v>
-      </c>
-      <c r="BD75" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="76" spans="1:58" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
-        <v>1541</v>
-      </c>
-      <c r="B76" t="s">
-        <v>1542</v>
-      </c>
-      <c r="C76" t="s">
-        <v>60</v>
-      </c>
-      <c r="D76" t="s">
-        <v>61</v>
-      </c>
-      <c r="F76" t="s">
-        <v>62</v>
-      </c>
-      <c r="G76" t="s">
-        <v>1543</v>
-      </c>
-      <c r="H76" t="s">
-        <v>1544</v>
-      </c>
-      <c r="I76" t="s">
-        <v>1545</v>
-      </c>
-      <c r="J76" t="s">
-        <v>176</v>
-      </c>
-      <c r="K76" t="s">
-        <v>1546</v>
-      </c>
-      <c r="L76" t="s">
-        <v>68</v>
-      </c>
-      <c r="M76" t="s">
-        <v>69</v>
-      </c>
-      <c r="N76" t="s">
-        <v>1547</v>
-      </c>
-      <c r="O76" t="s">
-        <v>1547</v>
-      </c>
-      <c r="P76" t="s">
-        <v>1548</v>
-      </c>
-      <c r="Q76" t="s">
-        <v>1549</v>
-      </c>
-      <c r="R76" t="s">
-        <v>1550</v>
-      </c>
-      <c r="S76" t="s">
-        <v>71</v>
-      </c>
-      <c r="T76" t="s">
-        <v>208</v>
-      </c>
-      <c r="U76" t="s">
-        <v>71</v>
-      </c>
-      <c r="V76" t="s">
-        <v>208</v>
-      </c>
-      <c r="X76" t="s">
-        <v>1550</v>
-      </c>
-      <c r="Y76" t="s">
-        <v>1551</v>
-      </c>
-      <c r="AC76" t="s">
-        <v>1552</v>
-      </c>
-      <c r="AD76" t="s">
-        <v>1553</v>
-      </c>
-      <c r="AE76" t="s">
-        <v>1554</v>
-      </c>
-      <c r="AI76" t="s">
-        <v>82</v>
-      </c>
-      <c r="AJ76" t="s">
-        <v>97</v>
-      </c>
-      <c r="AK76" t="s">
-        <v>1555</v>
-      </c>
-      <c r="AL76" t="s">
-        <v>85</v>
-      </c>
-      <c r="AM76" t="s">
-        <v>86</v>
-      </c>
-      <c r="AN76" t="s">
-        <v>134</v>
-      </c>
-      <c r="AO76" t="s">
-        <v>88</v>
-      </c>
-      <c r="AP76" t="s">
-        <v>1556</v>
-      </c>
-      <c r="AQ76" t="s">
-        <v>1557</v>
-      </c>
-      <c r="AR76" t="s">
-        <v>1558</v>
-      </c>
-      <c r="AS76" t="s">
-        <v>1559</v>
-      </c>
-      <c r="AT76" t="s">
-        <v>1560</v>
-      </c>
-      <c r="AU76" t="s">
-        <v>1561</v>
-      </c>
-      <c r="AV76" t="s">
-        <v>1562</v>
-      </c>
-      <c r="AW76" t="s">
-        <v>1563</v>
-      </c>
-      <c r="AX76" t="s">
-        <v>1561</v>
-      </c>
-      <c r="AY76" t="s">
-        <v>1564</v>
-      </c>
-      <c r="AZ76" t="s">
-        <v>166</v>
-      </c>
-      <c r="BA76" t="s">
-        <v>98</v>
-      </c>
-      <c r="BB76" t="s">
-        <v>1565</v>
-      </c>
-      <c r="BC76" t="s">
-        <v>1566</v>
-      </c>
-      <c r="BD76" t="s">
-        <v>1567</v>
-      </c>
-    </row>
-    <row r="77" spans="1:58" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
-        <v>1568</v>
-      </c>
-      <c r="B77" t="s">
-        <v>1569</v>
-      </c>
-      <c r="C77" t="s">
-        <v>60</v>
-      </c>
-      <c r="D77" t="s">
-        <v>61</v>
-      </c>
-      <c r="F77" t="s">
-        <v>62</v>
-      </c>
-      <c r="G77" t="s">
-        <v>1570</v>
-      </c>
-      <c r="H77" t="s">
-        <v>1571</v>
-      </c>
-      <c r="I77" t="s">
-        <v>1572</v>
-      </c>
-      <c r="J77" t="s">
-        <v>176</v>
-      </c>
-      <c r="K77" t="s">
-        <v>1573</v>
-      </c>
-      <c r="L77" t="s">
-        <v>68</v>
-      </c>
-      <c r="M77" t="s">
-        <v>69</v>
-      </c>
-      <c r="N77" t="s">
-        <v>1574</v>
-      </c>
-      <c r="O77" t="s">
-        <v>1574</v>
-      </c>
-      <c r="P77" t="s">
-        <v>1575</v>
-      </c>
-      <c r="Q77" t="s">
-        <v>1576</v>
-      </c>
-      <c r="R77" t="s">
-        <v>1577</v>
-      </c>
-      <c r="S77" t="s">
-        <v>1578</v>
-      </c>
-      <c r="T77" t="s">
-        <v>1579</v>
-      </c>
-      <c r="U77" t="s">
-        <v>71</v>
-      </c>
-      <c r="V77" t="s">
-        <v>1580</v>
-      </c>
-      <c r="X77" t="s">
-        <v>1581</v>
-      </c>
-      <c r="Y77" t="s">
-        <v>129</v>
-      </c>
-      <c r="AC77" t="s">
-        <v>1582</v>
-      </c>
-      <c r="AD77" t="s">
-        <v>379</v>
-      </c>
-      <c r="AE77" t="s">
-        <v>1583</v>
-      </c>
-      <c r="AI77" t="s">
-        <v>82</v>
-      </c>
-      <c r="AJ77" t="s">
-        <v>97</v>
-      </c>
-      <c r="AK77" t="s">
-        <v>1584</v>
-      </c>
-      <c r="AL77" t="s">
-        <v>85</v>
-      </c>
-      <c r="AM77" t="s">
-        <v>86</v>
-      </c>
-      <c r="AN77" t="s">
-        <v>1585</v>
-      </c>
-      <c r="AO77" t="s">
-        <v>88</v>
-      </c>
-      <c r="AP77" t="s">
-        <v>1586</v>
-      </c>
-      <c r="AQ77" t="s">
-        <v>1587</v>
-      </c>
-      <c r="AR77" t="s">
-        <v>1588</v>
-      </c>
-      <c r="AS77" t="s">
-        <v>1589</v>
-      </c>
-      <c r="AT77" t="s">
-        <v>1590</v>
-      </c>
-      <c r="AU77" t="s">
-        <v>1591</v>
-      </c>
-      <c r="AV77" t="s">
-        <v>1592</v>
-      </c>
-      <c r="AW77" t="s">
-        <v>389</v>
-      </c>
-      <c r="AX77" t="s">
-        <v>1591</v>
-      </c>
-      <c r="AY77" t="s">
-        <v>1593</v>
-      </c>
-      <c r="AZ77" t="s">
-        <v>1163</v>
-      </c>
-      <c r="BA77" t="s">
-        <v>98</v>
-      </c>
-      <c r="BB77" t="s">
-        <v>1594</v>
-      </c>
-      <c r="BC77" t="s">
-        <v>1595</v>
-      </c>
-      <c r="BD77" t="s">
-        <v>1567</v>
-      </c>
-    </row>
-    <row r="78" spans="1:58" x14ac:dyDescent="0.35">
-      <c r="A78" t="s">
-        <v>1596</v>
-      </c>
-      <c r="B78" t="s">
-        <v>1597</v>
-      </c>
-      <c r="C78" t="s">
-        <v>60</v>
-      </c>
-      <c r="D78" t="s">
-        <v>61</v>
-      </c>
-      <c r="F78" t="s">
-        <v>62</v>
-      </c>
-      <c r="G78" t="s">
-        <v>1598</v>
-      </c>
-      <c r="H78" t="s">
-        <v>1599</v>
-      </c>
-      <c r="I78" t="s">
-        <v>1600</v>
-      </c>
-      <c r="J78" t="s">
-        <v>176</v>
-      </c>
-      <c r="K78" t="s">
-        <v>1601</v>
-      </c>
-      <c r="L78" t="s">
-        <v>68</v>
-      </c>
-      <c r="M78" t="s">
-        <v>69</v>
-      </c>
-      <c r="N78" t="s">
-        <v>1602</v>
-      </c>
-      <c r="O78" t="s">
-        <v>1602</v>
-      </c>
-      <c r="P78" t="s">
-        <v>1603</v>
-      </c>
-      <c r="Q78" t="s">
-        <v>1604</v>
-      </c>
-      <c r="R78" t="s">
-        <v>1605</v>
-      </c>
-      <c r="S78" t="s">
-        <v>1606</v>
-      </c>
-      <c r="T78" t="s">
-        <v>635</v>
-      </c>
-      <c r="U78" t="s">
-        <v>71</v>
-      </c>
-      <c r="V78" t="s">
-        <v>76</v>
-      </c>
-      <c r="X78" t="s">
-        <v>1607</v>
-      </c>
-      <c r="Y78" t="s">
-        <v>129</v>
-      </c>
-      <c r="AC78" t="s">
-        <v>1608</v>
-      </c>
-      <c r="AD78" t="s">
-        <v>1609</v>
-      </c>
-      <c r="AE78" t="s">
-        <v>1610</v>
-      </c>
-      <c r="AI78" t="s">
-        <v>82</v>
-      </c>
-      <c r="AJ78" t="s">
-        <v>97</v>
-      </c>
-      <c r="AK78" t="s">
-        <v>1611</v>
-      </c>
-      <c r="AL78" t="s">
-        <v>85</v>
-      </c>
-      <c r="AM78" t="s">
-        <v>86</v>
-      </c>
-      <c r="AN78" t="s">
-        <v>1612</v>
-      </c>
-      <c r="AO78" t="s">
-        <v>88</v>
-      </c>
-      <c r="AP78" t="s">
-        <v>1613</v>
-      </c>
-      <c r="AQ78" t="s">
-        <v>1614</v>
-      </c>
-      <c r="AR78" t="s">
-        <v>1615</v>
-      </c>
-      <c r="AS78" t="s">
-        <v>1616</v>
-      </c>
-      <c r="AT78" t="s">
-        <v>1617</v>
-      </c>
-      <c r="AU78" t="s">
-        <v>1618</v>
-      </c>
-      <c r="AV78" t="s">
-        <v>1619</v>
-      </c>
-      <c r="AW78" t="s">
-        <v>142</v>
-      </c>
-      <c r="AX78" t="s">
-        <v>1620</v>
-      </c>
-      <c r="AY78" t="s">
-        <v>1621</v>
-      </c>
-      <c r="AZ78" t="s">
-        <v>649</v>
-      </c>
-      <c r="BA78" t="s">
-        <v>98</v>
-      </c>
-      <c r="BB78" t="s">
-        <v>1622</v>
-      </c>
-      <c r="BC78" t="s">
-        <v>1623</v>
-      </c>
-      <c r="BD78" t="s">
-        <v>1567</v>
-      </c>
-    </row>
-    <row r="79" spans="1:58" x14ac:dyDescent="0.35">
-      <c r="A79" t="s">
-        <v>1624</v>
-      </c>
-      <c r="C79" t="s">
-        <v>350</v>
-      </c>
-      <c r="D79" t="s">
-        <v>350</v>
-      </c>
-      <c r="E79" t="s">
-        <v>351</v>
-      </c>
-      <c r="F79" t="s">
-        <v>62</v>
-      </c>
-      <c r="G79" t="s">
-        <v>1598</v>
-      </c>
-      <c r="H79" t="s">
-        <v>1599</v>
-      </c>
-      <c r="I79" t="s">
-        <v>1600</v>
-      </c>
-      <c r="J79" t="s">
-        <v>176</v>
-      </c>
-      <c r="K79" t="s">
-        <v>1601</v>
-      </c>
-      <c r="L79" t="s">
-        <v>68</v>
-      </c>
-      <c r="M79" t="s">
-        <v>68</v>
-      </c>
-      <c r="N79" t="s">
-        <v>1602</v>
-      </c>
-      <c r="O79" t="s">
-        <v>1602</v>
-      </c>
-      <c r="P79" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q79" t="s">
-        <v>1604</v>
-      </c>
-      <c r="R79" t="s">
-        <v>1625</v>
-      </c>
-      <c r="S79" t="s">
-        <v>1606</v>
-      </c>
-      <c r="T79" t="s">
-        <v>635</v>
-      </c>
-      <c r="U79" t="s">
-        <v>71</v>
-      </c>
-      <c r="V79" t="s">
-        <v>76</v>
-      </c>
-      <c r="X79" t="s">
-        <v>1626</v>
-      </c>
-      <c r="Y79" t="s">
-        <v>129</v>
-      </c>
-      <c r="Z79" t="s">
-        <v>1625</v>
-      </c>
-      <c r="AA79" t="s">
-        <v>420</v>
-      </c>
-      <c r="AB79" t="s">
-        <v>421</v>
-      </c>
-      <c r="AC79" t="s">
-        <v>1627</v>
-      </c>
-      <c r="AH79" t="s">
-        <v>1628</v>
-      </c>
-      <c r="AI79" t="s">
-        <v>82</v>
-      </c>
-      <c r="AJ79" t="s">
-        <v>97</v>
-      </c>
-      <c r="AL79" t="s">
-        <v>85</v>
-      </c>
-      <c r="AM79" t="s">
-        <v>86</v>
-      </c>
-      <c r="AN79" t="s">
-        <v>1612</v>
-      </c>
-      <c r="AP79" t="s">
-        <v>1613</v>
-      </c>
-      <c r="AQ79" t="s">
-        <v>1614</v>
-      </c>
-      <c r="AR79" t="s">
-        <v>1615</v>
-      </c>
-      <c r="AS79" t="s">
-        <v>1629</v>
-      </c>
-      <c r="AT79" t="s">
-        <v>1617</v>
-      </c>
-      <c r="AU79" t="s">
-        <v>486</v>
-      </c>
-      <c r="AV79" t="s">
-        <v>370</v>
-      </c>
-      <c r="AW79" t="s">
-        <v>1311</v>
-      </c>
-      <c r="AX79" t="s">
-        <v>371</v>
-      </c>
-      <c r="AY79" t="s">
-        <v>1621</v>
-      </c>
-      <c r="AZ79" t="s">
-        <v>649</v>
-      </c>
-      <c r="BA79" t="s">
-        <v>98</v>
-      </c>
-      <c r="BB79" t="s">
-        <v>373</v>
-      </c>
-      <c r="BC79" t="s">
-        <v>1630</v>
-      </c>
-    </row>
-    <row r="80" spans="1:58" x14ac:dyDescent="0.35">
-      <c r="A80" t="s">
-        <v>1631</v>
-      </c>
-      <c r="C80" t="s">
-        <v>350</v>
-      </c>
-      <c r="D80" t="s">
-        <v>350</v>
-      </c>
-      <c r="E80" t="s">
-        <v>351</v>
-      </c>
-      <c r="F80" t="s">
-        <v>62</v>
-      </c>
-      <c r="G80" t="s">
-        <v>1632</v>
-      </c>
-      <c r="H80" t="s">
-        <v>1633</v>
-      </c>
-      <c r="I80" t="s">
-        <v>1634</v>
-      </c>
-      <c r="J80" t="s">
-        <v>176</v>
-      </c>
-      <c r="K80" t="s">
-        <v>1635</v>
-      </c>
-      <c r="L80" t="s">
-        <v>68</v>
-      </c>
-      <c r="M80" t="s">
-        <v>68</v>
-      </c>
-      <c r="N80" t="s">
-        <v>1636</v>
-      </c>
-      <c r="O80" t="s">
-        <v>1636</v>
-      </c>
-      <c r="P80" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q80" t="s">
-        <v>1637</v>
-      </c>
-      <c r="R80" t="s">
-        <v>1638</v>
-      </c>
-      <c r="S80" t="s">
-        <v>126</v>
-      </c>
-      <c r="T80" t="s">
-        <v>127</v>
-      </c>
-      <c r="U80" t="s">
-        <v>71</v>
-      </c>
-      <c r="V80" t="s">
-        <v>76</v>
-      </c>
-      <c r="X80" t="s">
-        <v>1639</v>
-      </c>
-      <c r="Y80" t="s">
-        <v>129</v>
-      </c>
-      <c r="Z80" t="s">
-        <v>1638</v>
-      </c>
-      <c r="AA80" t="s">
-        <v>360</v>
-      </c>
-      <c r="AB80" t="s">
-        <v>554</v>
-      </c>
-      <c r="AC80" t="s">
-        <v>1640</v>
-      </c>
-      <c r="AH80" t="s">
-        <v>1641</v>
-      </c>
-      <c r="AI80" t="s">
-        <v>82</v>
-      </c>
-      <c r="AJ80" t="s">
-        <v>97</v>
-      </c>
-      <c r="AL80" t="s">
-        <v>85</v>
-      </c>
-      <c r="AM80" t="s">
-        <v>86</v>
-      </c>
-      <c r="AN80" t="s">
-        <v>134</v>
-      </c>
-      <c r="AP80" t="s">
-        <v>1642</v>
-      </c>
-      <c r="AQ80" t="s">
-        <v>1643</v>
-      </c>
-      <c r="AR80" t="s">
-        <v>1644</v>
-      </c>
-      <c r="AS80" t="s">
-        <v>1645</v>
-      </c>
-      <c r="AT80" t="s">
-        <v>1646</v>
-      </c>
-      <c r="AU80" t="s">
-        <v>429</v>
-      </c>
-      <c r="AV80" t="s">
-        <v>487</v>
-      </c>
-      <c r="AW80" t="s">
-        <v>369</v>
-      </c>
-      <c r="AX80" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AY80" t="s">
-        <v>1648</v>
-      </c>
-      <c r="AZ80" t="s">
-        <v>451</v>
-      </c>
-      <c r="BA80" t="s">
-        <v>98</v>
-      </c>
-      <c r="BB80" t="s">
-        <v>373</v>
-      </c>
-      <c r="BC80" t="s">
-        <v>1649</v>
       </c>
     </row>
   </sheetData>

</xml_diff>